<commit_message>
Mise a jour automatique 18/10/2026 19:24:27,69
</commit_message>
<xml_diff>
--- a/data/resultats/resultats.xlsx
+++ b/data/resultats/resultats.xlsx
@@ -50,6 +50,39 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>DMU11-8</t>
+  </si>
+  <si>
+    <t>28523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BREBIERES BC (6) </t>
+  </si>
+  <si>
+    <t>17/10/2026</t>
+  </si>
+  <si>
+    <t>15:30</t>
+  </si>
+  <si>
+    <t>JEAN DEGROS</t>
+  </si>
+  <si>
+    <t>9UDZ2ZGP</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
     <t>DFU15-8</t>
   </si>
   <si>
@@ -62,24 +95,12 @@
     <t xml:space="preserve">BREBIERES BC (4) </t>
   </si>
   <si>
-    <t>17/10/2026</t>
-  </si>
-  <si>
     <t>17:00</t>
   </si>
   <si>
-    <t>JEAN DEGROS</t>
-  </si>
-  <si>
     <t>A4A44MUC</t>
   </si>
   <si>
-    <t>45</t>
-  </si>
-  <si>
-    <t>Non</t>
-  </si>
-  <si>
     <t>35</t>
   </si>
   <si>
@@ -89,9 +110,6 @@
     <t>29323</t>
   </si>
   <si>
-    <t xml:space="preserve">BREBIERES BC (6) </t>
-  </si>
-  <si>
     <t>14:00</t>
   </si>
   <si>
@@ -104,22 +122,28 @@
     <t>10</t>
   </si>
   <si>
-    <t>DMU11-8</t>
-  </si>
-  <si>
-    <t>28523</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (5) </t>
-  </si>
-  <si>
-    <t>15:30</t>
-  </si>
-  <si>
-    <t>9UDZ2ZGP</t>
-  </si>
-  <si>
-    <t>16</t>
+    <t>DFU18-2</t>
+  </si>
+  <si>
+    <t>7011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT - 2 (1) </t>
+  </si>
+  <si>
+    <t>20:30</t>
+  </si>
+  <si>
+    <t>64Y8HJ6Y</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>80</t>
   </si>
   <si>
     <t>DMU15-2</t>
@@ -143,6 +167,30 @@
     <t>73</t>
   </si>
   <si>
+    <t>DM2</t>
+  </si>
+  <si>
+    <t>689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUINCY ASB (4) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (2) </t>
+  </si>
+  <si>
+    <t>Jean LENNE</t>
+  </si>
+  <si>
+    <t>TYQDQK3L</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
     <t>DFU9-8</t>
   </si>
   <si>
@@ -158,39 +206,12 @@
     <t>12</t>
   </si>
   <si>
-    <t>DM2</t>
-  </si>
-  <si>
-    <t>689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUINCY ASB (4) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 2 (2) </t>
-  </si>
-  <si>
-    <t>Jean LENNE</t>
-  </si>
-  <si>
-    <t>TYQDQK3L</t>
-  </si>
-  <si>
-    <t>48</t>
-  </si>
-  <si>
-    <t>63</t>
-  </si>
-  <si>
     <t>PRM</t>
   </si>
   <si>
     <t>112</t>
   </si>
   <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT - 2 (3) </t>
-  </si>
-  <si>
     <t xml:space="preserve">AMICALE BASKET PECQUENCOURT - 1 (5) </t>
   </si>
   <si>
@@ -206,7 +227,10 @@
     <t>VLPR4CMA</t>
   </si>
   <si>
-    <t/>
+    <t>54</t>
+  </si>
+  <si>
+    <t>52</t>
   </si>
   <si>
     <t>DMU18-2</t>
@@ -245,9 +269,6 @@
     <t>JBJGRZMN</t>
   </si>
   <si>
-    <t>51</t>
-  </si>
-  <si>
     <t>27</t>
   </si>
   <si>
@@ -294,27 +315,6 @@
   </si>
   <si>
     <t>25</t>
-  </si>
-  <si>
-    <t>DFU18-2</t>
-  </si>
-  <si>
-    <t>7011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT - 2 (1) </t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>64Y8HJ6Y</t>
-  </si>
-  <si>
-    <t>80</t>
   </si>
 </sst>
 </file>
@@ -461,25 +461,25 @@
         <v>24</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s" s="0">
         <v>18</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="J3" t="s" s="0">
         <v>21</v>
@@ -499,25 +499,25 @@
         <v>31</v>
       </c>
       <c r="C4" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F4" t="s" s="0">
         <v>32</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F4" t="s" s="0">
-        <v>33</v>
       </c>
       <c r="G4" t="s" s="0">
         <v>18</v>
       </c>
       <c r="H4" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="I4" t="s" s="0">
         <v>34</v>
-      </c>
-      <c r="I4" t="s" s="0">
-        <v>20</v>
       </c>
       <c r="J4" t="s" s="0">
         <v>21</v>
@@ -537,31 +537,31 @@
         <v>37</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G5" t="s" s="0">
         <v>18</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J5" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L5" t="s" s="0">
         <v>21</v>
@@ -569,37 +569,37 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>14</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="J6" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="L6" t="s" s="0">
         <v>21</v>
@@ -607,37 +607,37 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="J7" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L7" t="s" s="0">
         <v>21</v>
@@ -645,37 +645,37 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="F8" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="G8" t="s" s="0">
         <v>61</v>
       </c>
-      <c r="G8" t="s" s="0">
+      <c r="H8" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="H8" t="s" s="0">
+      <c r="I8" t="s" s="0">
         <v>63</v>
       </c>
-      <c r="I8" t="s" s="0">
-        <v>64</v>
-      </c>
       <c r="J8" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K8" t="s" s="0">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="L8" t="s" s="0">
         <v>21</v>
@@ -683,37 +683,37 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="B9" t="s" s="0">
         <v>65</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="C9" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D9" t="s" s="0">
         <v>66</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="E9" t="s" s="0">
         <v>67</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>32</v>
-      </c>
-      <c r="E9" t="s" s="0">
-        <v>16</v>
-      </c>
       <c r="F9" t="s" s="0">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I9" t="s" s="0">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J9" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K9" t="s" s="0">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L9" t="s" s="0">
         <v>21</v>
@@ -721,37 +721,37 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J10" t="s" s="0">
         <v>21</v>
       </c>
       <c r="K10" t="s" s="0">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L10" t="s" s="0">
         <v>21</v>
@@ -759,22 +759,22 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>82</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s" s="0">
         <v>83</v>
@@ -783,13 +783,13 @@
         <v>84</v>
       </c>
       <c r="I11" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="J11" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="K11" t="s" s="0">
         <v>85</v>
-      </c>
-      <c r="J11" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="K11" t="s" s="0">
-        <v>28</v>
       </c>
       <c r="L11" t="s" s="0">
         <v>21</v>
@@ -806,13 +806,13 @@
         <v>88</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="G12" t="s" s="0">
         <v>90</v>
@@ -827,7 +827,7 @@
         <v>21</v>
       </c>
       <c r="K12" t="s" s="0">
-        <v>93</v>
+        <v>34</v>
       </c>
       <c r="L12" t="s" s="0">
         <v>21</v>
@@ -835,31 +835,31 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
+        <v>93</v>
+      </c>
+      <c r="B13" t="s" s="0">
         <v>94</v>
       </c>
-      <c r="B13" t="s" s="0">
+      <c r="C13" t="s" s="0">
         <v>95</v>
       </c>
-      <c r="C13" t="s" s="0">
+      <c r="D13" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="F13" t="s" s="0">
         <v>96</v>
       </c>
-      <c r="D13" t="s" s="0">
+      <c r="G13" t="s" s="0">
         <v>97</v>
       </c>
-      <c r="E13" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F13" t="s" s="0">
+      <c r="H13" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="G13" t="s" s="0">
-        <v>18</v>
-      </c>
-      <c r="H13" t="s" s="0">
+      <c r="I13" t="s" s="0">
         <v>99</v>
-      </c>
-      <c r="I13" t="s" s="0">
-        <v>77</v>
       </c>
       <c r="J13" t="s" s="0">
         <v>21</v>

</xml_diff>